<commit_message>
corpus: reconversia orașelor cu cache de extracție expirat (10 din 11)
Reconvertite cu pipeline-ul curent, apoi trecute prin detecția reparată
a totalurilor: 20 de orașe au acum totalul de venituri (față de 15), 11
pe cel de cheltuieli, iar comparația execuție-vs-plan acoperă 18 (față
de 13). Buzău primește un infografic complet.

Bistrița a rămas la conversia anterioară: extracția curentă îi pierde 70
de linii verificate fără să câștige vreun total — singura pierdere netă
din serie. Scăderile de procent la Galați, Miercurea Ciuc, Focșani și
Alexandria sunt aparente: numărul absolut de linii verificate e neschimbat,
doar că extractorul citește acum mai multe rânduri pe care le marchează.

Buzău e un compromis asumat: pierde linii verificate, dar câștigă ambele
totaluri — 43,5% și 37,3% din execuția Forexebug, echilibrate între ele,
deci confirmate de o sursă independentă.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/2026/41-vrancea/174744-focsani/budget_file.xlsx
+++ b/data/2026/41-vrancea/174744-focsani/budget_file.xlsx
@@ -3199,38 +3199,49 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>03.02</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="n"/>
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>Impozit teren extravilan</t>
         </is>
       </c>
-      <c r="E78" t="n">
+      <c r="D78" s="4" t="n"/>
+      <c r="E78" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" s="3" t="n"/>
-      <c r="H78" s="3" t="n">
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="n"/>
+      <c r="H78" s="5" t="n">
         <v>310</v>
       </c>
-      <c r="I78" s="3" t="n"/>
-      <c r="J78" s="3" t="n"/>
-      <c r="K78" s="3" t="n"/>
-      <c r="L78" s="3" t="n"/>
-      <c r="M78" s="3" t="n"/>
-      <c r="N78" s="3" t="n"/>
-      <c r="O78" s="3" t="n"/>
-      <c r="P78" s="3" t="n"/>
-      <c r="Q78" s="3" t="n"/>
-      <c r="R78" s="3" t="n"/>
-      <c r="S78" s="3" t="n"/>
-      <c r="T78" t="inlineStr">
-        <is>
-          <t>ocr</t>
+      <c r="I78" s="5" t="n"/>
+      <c r="J78" s="5" t="n"/>
+      <c r="K78" s="5" t="n"/>
+      <c r="L78" s="5" t="n"/>
+      <c r="M78" s="5" t="n"/>
+      <c r="N78" s="5" t="n"/>
+      <c r="O78" s="5" t="n"/>
+      <c r="P78" s="5" t="n"/>
+      <c r="Q78" s="5" t="n"/>
+      <c r="R78" s="5" t="n"/>
+      <c r="S78" s="5" t="n"/>
+      <c r="T78" s="4" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="U78" s="4" t="inlineStr">
+        <is>
+          <t>03.02 total_2026: parent 310,00 != sum(children) 2,03 (1 children)</t>
         </is>
       </c>
     </row>
@@ -17422,38 +17433,49 @@
       </c>
     </row>
     <row r="439">
-      <c r="A439" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="C439" s="2" t="inlineStr">
+      <c r="A439" s="6" t="inlineStr">
+        <is>
+          <t>31.02</t>
+        </is>
+      </c>
+      <c r="B439" s="6" t="n"/>
+      <c r="C439" s="6" t="inlineStr">
         <is>
           <t>(materiale dendrologice, ingrasaminte, unelte grădinărit, cosit gazon, tuns gard viu, toaletari copaci,costuri utilaje-carburanti, piese de schimb, utilități sere,etc) varsaminte la bugetul de stat aferent persoane cu handicap neincadrate</t>
         </is>
       </c>
-      <c r="E439" t="n">
+      <c r="D439" s="6" t="n"/>
+      <c r="E439" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F439" t="inlineStr"/>
-      <c r="G439" s="3" t="n"/>
-      <c r="H439" s="3" t="n">
+      <c r="F439" s="6" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="G439" s="7" t="n"/>
+      <c r="H439" s="7" t="n">
         <v>31</v>
       </c>
-      <c r="I439" s="3" t="n"/>
-      <c r="J439" s="3" t="n"/>
-      <c r="K439" s="3" t="n"/>
-      <c r="L439" s="3" t="n"/>
-      <c r="M439" s="3" t="n"/>
-      <c r="N439" s="3" t="n"/>
-      <c r="O439" s="3" t="n"/>
-      <c r="P439" s="3" t="n"/>
-      <c r="Q439" s="3" t="n"/>
-      <c r="R439" s="3" t="n"/>
-      <c r="S439" s="3" t="n"/>
-      <c r="T439" t="inlineStr">
-        <is>
-          <t>ocr</t>
+      <c r="I439" s="7" t="n"/>
+      <c r="J439" s="7" t="n"/>
+      <c r="K439" s="7" t="n"/>
+      <c r="L439" s="7" t="n"/>
+      <c r="M439" s="7" t="n"/>
+      <c r="N439" s="7" t="n"/>
+      <c r="O439" s="7" t="n"/>
+      <c r="P439" s="7" t="n"/>
+      <c r="Q439" s="7" t="n"/>
+      <c r="R439" s="7" t="n"/>
+      <c r="S439" s="7" t="n"/>
+      <c r="T439" s="6" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="U439" s="6" t="inlineStr">
+        <is>
+          <t>name mismatch vs nomenclator (13%): '(materiale dendrologice, ingrasaminte, u' vs 'Venituri din dobanzi'</t>
         </is>
       </c>
     </row>
@@ -17522,74 +17544,96 @@
       </c>
     </row>
     <row r="442">
-      <c r="A442" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="C442" s="2" t="inlineStr">
+      <c r="A442" s="6" t="inlineStr">
+        <is>
+          <t>35.02</t>
+        </is>
+      </c>
+      <c r="B442" s="6" t="n"/>
+      <c r="C442" s="6" t="inlineStr">
         <is>
           <t>iluminat public</t>
         </is>
       </c>
-      <c r="E442" t="n">
+      <c r="D442" s="6" t="n"/>
+      <c r="E442" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F442" t="inlineStr"/>
-      <c r="G442" s="3" t="n"/>
-      <c r="H442" s="3" t="n">
+      <c r="F442" s="6" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="G442" s="7" t="n"/>
+      <c r="H442" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="I442" s="3" t="n"/>
-      <c r="J442" s="3" t="n"/>
-      <c r="K442" s="3" t="n"/>
-      <c r="L442" s="3" t="n"/>
-      <c r="M442" s="3" t="n"/>
-      <c r="N442" s="3" t="n"/>
-      <c r="O442" s="3" t="n"/>
-      <c r="P442" s="3" t="n"/>
-      <c r="Q442" s="3" t="n"/>
-      <c r="R442" s="3" t="n"/>
-      <c r="S442" s="3" t="n"/>
-      <c r="T442" t="inlineStr">
-        <is>
-          <t>ocr</t>
+      <c r="I442" s="7" t="n"/>
+      <c r="J442" s="7" t="n"/>
+      <c r="K442" s="7" t="n"/>
+      <c r="L442" s="7" t="n"/>
+      <c r="M442" s="7" t="n"/>
+      <c r="N442" s="7" t="n"/>
+      <c r="O442" s="7" t="n"/>
+      <c r="P442" s="7" t="n"/>
+      <c r="Q442" s="7" t="n"/>
+      <c r="R442" s="7" t="n"/>
+      <c r="S442" s="7" t="n"/>
+      <c r="T442" s="6" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="U442" s="6" t="inlineStr">
+        <is>
+          <t>name mismatch vs nomenclator (34%): 'iluminat public' vs 'Amenzi, penalitati si confiscari'</t>
         </is>
       </c>
     </row>
     <row r="443">
-      <c r="A443" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="C443" s="2" t="inlineStr">
+      <c r="A443" s="6" t="inlineStr">
+        <is>
+          <t>35.02</t>
+        </is>
+      </c>
+      <c r="B443" s="6" t="n"/>
+      <c r="C443" s="6" t="inlineStr">
         <is>
           <t>materiale intretinere iluminat</t>
         </is>
       </c>
-      <c r="E443" t="n">
+      <c r="D443" s="6" t="n"/>
+      <c r="E443" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F443" t="inlineStr"/>
-      <c r="G443" s="3" t="n"/>
-      <c r="H443" s="3" t="n">
+      <c r="F443" s="6" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="G443" s="7" t="n"/>
+      <c r="H443" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="I443" s="3" t="n"/>
-      <c r="J443" s="3" t="n"/>
-      <c r="K443" s="3" t="n"/>
-      <c r="L443" s="3" t="n"/>
-      <c r="M443" s="3" t="n"/>
-      <c r="N443" s="3" t="n"/>
-      <c r="O443" s="3" t="n"/>
-      <c r="P443" s="3" t="n"/>
-      <c r="Q443" s="3" t="n"/>
-      <c r="R443" s="3" t="n"/>
-      <c r="S443" s="3" t="n"/>
-      <c r="T443" t="inlineStr">
-        <is>
-          <t>ocr</t>
+      <c r="I443" s="7" t="n"/>
+      <c r="J443" s="7" t="n"/>
+      <c r="K443" s="7" t="n"/>
+      <c r="L443" s="7" t="n"/>
+      <c r="M443" s="7" t="n"/>
+      <c r="N443" s="7" t="n"/>
+      <c r="O443" s="7" t="n"/>
+      <c r="P443" s="7" t="n"/>
+      <c r="Q443" s="7" t="n"/>
+      <c r="R443" s="7" t="n"/>
+      <c r="S443" s="7" t="n"/>
+      <c r="T443" s="6" t="inlineStr">
+        <is>
+          <t>ocr</t>
+        </is>
+      </c>
+      <c r="U443" s="6" t="inlineStr">
+        <is>
+          <t>name mismatch vs nomenclator (35%): 'materiale intretinere iluminat' vs 'Amenzi, penalitati si confiscari'</t>
         </is>
       </c>
     </row>
@@ -28266,7 +28310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -28325,7 +28369,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>16.02</t>
+          <t>03.02</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -28335,7 +28379,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LLM re-read 4 rows for 16.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>LLM re-read 2 rows for 03.02 total_2026: still inconsistent — UNRESOLVED</t>
         </is>
       </c>
     </row>
@@ -28351,11 +28395,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>35.02</t>
+          <t>16.02</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -28365,7 +28409,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>LLM re-read 3 rows for 35.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>LLM re-read 4 rows for 16.02 total_2026: still inconsistent — UNRESOLVED</t>
         </is>
       </c>
     </row>
@@ -28385,7 +28429,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>11.02</t>
+          <t>35.02</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -28395,7 +28439,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>LLM re-read 4 rows for 11.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>LLM re-read 3 rows for 35.02 total_2026: still inconsistent — UNRESOLVED</t>
         </is>
       </c>
     </row>
@@ -28415,7 +28459,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>42.02</t>
+          <t>11.02</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -28425,7 +28469,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>LLM re-read 3 rows for 42.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>LLM re-read 4 rows for 11.02 total_2026: still inconsistent — UNRESOLVED</t>
         </is>
       </c>
     </row>
@@ -28441,11 +28485,11 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>61.02</t>
+          <t>42.02</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -28455,7 +28499,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LLM re-read 2 rows for 61.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>LLM re-read 3 rows for 42.02 total_2026: still inconsistent — UNRESOLVED</t>
         </is>
       </c>
     </row>
@@ -28471,11 +28515,11 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>66.02</t>
+          <t>61.02</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -28485,7 +28529,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LLM re-read 2 rows for 66.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>LLM re-read 2 rows for 61.02 total_2026: still inconsistent — UNRESOLVED</t>
         </is>
       </c>
     </row>
@@ -28505,7 +28549,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>68.02</t>
+          <t>66.02</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -28515,7 +28559,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>LLM re-read 3 rows for 68.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>LLM re-read 2 rows for 66.02 total_2026: still inconsistent — UNRESOLVED</t>
         </is>
       </c>
     </row>
@@ -28531,11 +28575,11 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>74.02</t>
+          <t>68.02</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -28545,7 +28589,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>LLM re-read 2 rows for 74.02 total_2026: still inconsistent — UNRESOLVED</t>
+          <t>LLM re-read 3 rows for 68.02 total_2026: still inconsistent — UNRESOLVED</t>
         </is>
       </c>
     </row>
@@ -28557,15 +28601,25 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>74.02</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>total_2026</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>unparseable-cell pass p5: 0 cells recovered</t>
+          <t>LLM re-read 2 rows for 74.02 total_2026: still inconsistent — UNRESOLVED</t>
         </is>
       </c>
     </row>
@@ -28581,11 +28635,11 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>unparseable-cell pass p6: 1 cells recovered</t>
+          <t>unparseable-cell pass p5: 0 cells recovered</t>
         </is>
       </c>
     </row>
@@ -28601,11 +28655,11 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>unparseable-cell pass p15: 0 cells recovered</t>
+          <t>unparseable-cell pass p6: 1 cells recovered</t>
         </is>
       </c>
     </row>
@@ -28621,41 +28675,31 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>unparseable-cell pass p24: 8 cells recovered</t>
+          <t>unparseable-cell pass p15: 0 cells recovered</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V6_repair</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>info</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>16.02</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>total_2026</t>
-        </is>
+        <v>24</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>16.02 total_2026: parent 12,59 != sum(children) 90,51 (3 children)</t>
+          <t>unparseable-cell pass p24: 8 cells recovered</t>
         </is>
       </c>
     </row>
@@ -28671,11 +28715,11 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>35.02</t>
+          <t>03.02</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -28685,7 +28729,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>35.02 total_2026: parent 4,09 != sum(children) 967,12 (2 children)</t>
+          <t>03.02 total_2026: parent 310,00 != sum(children) 2,03 (1 children)</t>
         </is>
       </c>
     </row>
@@ -28701,11 +28745,11 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>11.02</t>
+          <t>16.02</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -28715,7 +28759,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>11.02 total_2026: parent 69,26 != sum(children) 169,16 (3 children)</t>
+          <t>16.02 total_2026: parent 12,59 != sum(children) 90,51 (3 children)</t>
         </is>
       </c>
     </row>
@@ -28735,7 +28779,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>42.02</t>
+          <t>35.02</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -28745,19 +28789,19 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>42.02 total_2026: parent 11,75 != sum(children) 261,50 (2 children)</t>
+          <t>35.02 total_2026: parent 4,09 != sum(children) 967,12 (2 children)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -28765,24 +28809,29 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>42.02</t>
+          <t>11.02</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (55%): 'SUBVENTII PENTRU INVESTITII' vs 'Subventii de la bugetul de stat'</t>
+          <t>11.02 total_2026: parent 69,26 != sum(children) 169,16 (3 children)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -28790,12 +28839,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>42.02.69</t>
+          <t>42.02</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (36%): 'Sume BS cofinantare proiecte UE 2014-202' vs 'Subvenţii de la bugetul de stat către bu'</t>
+          <t>42.02 total_2026: parent 11,75 != sum(children) 261,50 (2 children)</t>
         </is>
       </c>
     </row>
@@ -28815,12 +28869,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>42.02.93</t>
+          <t>42.02</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (51%): 'Sume BS cofinantare proiecte UE 2021-202' vs 'Subvenţii de la bugetul de stat necesare'</t>
+          <t>name mismatch vs nomenclator (55%): 'SUBVENTII PENTRU INVESTITII' vs 'Subventii de la bugetul de stat'</t>
         </is>
       </c>
     </row>
@@ -28840,12 +28894,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>42.02.65</t>
+          <t>42.02.69</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Finanţarea Programului Naţional de Dezvo'</t>
+          <t>name mismatch vs nomenclator (36%): 'Sume BS cofinantare proiecte UE 2014-202' vs 'Subvenţii de la bugetul de stat către bu'</t>
         </is>
       </c>
     </row>
@@ -28865,12 +28919,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>45.02</t>
+          <t>42.02.93</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (50%): 'SUME DE PRIMIT DE LA UE 2021-2027' vs 'Sume primite de la UE/alti donatori în c'</t>
+          <t>name mismatch vs nomenclator (51%): 'Sume BS cofinantare proiecte UE 2021-202' vs 'Subvenţii de la bugetul de stat necesare'</t>
         </is>
       </c>
     </row>
@@ -28886,41 +28940,41 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>42.02.65</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (28%): 'cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Finanţarea Programului Naţional de Dezvo'</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>4</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>45.02</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>unparseable cell '2,115 1,000' in column total_2026</t>
+          <t>name mismatch vs nomenclator (50%): 'SUME DE PRIMIT DE LA UE 2021-2027' vs 'Sume primite de la UE/alti donatori în c'</t>
         </is>
       </c>
     </row>
@@ -28940,49 +28994,49 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>54.02.07</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (43%): '*Fond de rezerva bugetara *Fond pt.garan' vs 'Fond pentru garantarea împrumuturilor ex'</t>
+          <t>name mismatch vs nomenclator (28%): 'cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>5</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>55.02</t>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (25%): 'Dobanzi' vs 'Tranzactii privind datoria publica si im'</t>
+          <t>unparseable cell '2,115 1,000' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -28990,17 +29044,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>61.02</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>54.02.07</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>61.02 total_2026: parent 9,99 != sum(children) 180,00 (1 children)</t>
+          <t>name mismatch vs nomenclator (43%): '*Fond de rezerva bugetara *Fond pt.garan' vs 'Fond pentru garantarea împrumuturilor ex'</t>
         </is>
       </c>
     </row>
@@ -29020,24 +29069,24 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>55.02</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (33%): '_cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
+          <t>name mismatch vs nomenclator (25%): 'Dobanzi' vs 'Tranzactii privind datoria publica si im'</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -29045,12 +29094,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>61.02.05</t>
+          <t>61.02</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (52%): '*Protectia civila' vs 'Protectie civila si protectia contra inc'</t>
+          <t>61.02 total_2026: parent 9,99 != sum(children) 180,00 (1 children)</t>
         </is>
       </c>
     </row>
@@ -29075,37 +29129,32 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (28%): 'cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
+          <t>name mismatch vs nomenclator (33%): '_cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>66.02</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>61.02.05</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>66.02 total_2026: parent 11,99 != sum(children) 11,96 (1 children)</t>
+          <t>name mismatch vs nomenclator (52%): '*Protectia civila' vs 'Protectie civila si protectia contra inc'</t>
         </is>
       </c>
     </row>
@@ -29121,7 +29170,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -29137,12 +29186,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -29150,12 +29199,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>66.02</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>duplicate of p6 with different values</t>
+          <t>66.02 total_2026: parent 11,99 != sum(children) 11,96 (1 children)</t>
         </is>
       </c>
     </row>
@@ -29187,12 +29241,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -29200,17 +29254,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>68.02</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>51</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>68.02 total_2026: parent 70,32 != sum(children) 34,32 (2 children)</t>
+          <t>duplicate of p6 with different values</t>
         </is>
       </c>
     </row>
@@ -29235,19 +29284,19 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (33%): '_cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
+          <t>name mismatch vs nomenclator (28%): 'cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>info</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -29255,7 +29304,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>70.02.10</t>
+          <t>68.02</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -29265,7 +29314,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>68.02 total_2026: parent 70,32 != sum(children) 34,32 (2 children)</t>
         </is>
       </c>
     </row>
@@ -29290,27 +29339,27 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (28%): 'cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
+          <t>name mismatch vs nomenclator (33%): '_cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>V4_hierarchy</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V6_repair</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>info</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>74.02</t>
+          <t>70.02.10</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -29320,7 +29369,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>74.02 total_2026: parent 15,78 != sum(children) 450,00 (1 children)</t>
+          <t>cell re-read from image (unverified transcription)</t>
         </is>
       </c>
     </row>
@@ -29336,7 +29385,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -29352,12 +29401,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V4_hierarchy</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -29365,12 +29414,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>74.02</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (38%): 'operatiuni financiare' vs 'TITLUL XX RAMBURSARI DE CREDITE'</t>
+          <t>74.02 total_2026: parent 15,78 != sum(children) 450,00 (1 children)</t>
         </is>
       </c>
     </row>
@@ -29395,7 +29449,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (33%): '_cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
+          <t>name mismatch vs nomenclator (28%): 'cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
         </is>
       </c>
     </row>
@@ -29415,12 +29469,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>81</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (41%): 'participare la capitalul social al socie' vs 'TITLUL XVII ACTIVE FINANCIARE'</t>
+          <t>name mismatch vs nomenclator (38%): 'operatiuni financiare' vs 'TITLUL XX RAMBURSARI DE CREDITE'</t>
         </is>
       </c>
     </row>
@@ -29477,100 +29531,100 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>8</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>7</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>71</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>unparseable cell 'VENITURI' in column total_2026</t>
+          <t>name mismatch vs nomenclator (33%): '_cheltuieli de capital' vs 'TITLUL XVI ACTIVE NEFINANCIARE (71.01+71'</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>8</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>est2027</t>
+        <v>7</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>72</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>unparseable cell 'Venituri operationale' in column est2027</t>
+          <t>name mismatch vs nomenclator (41%): 'participare la capitalul social al socie' vs 'TITLUL XVII ACTIVE FINANCIARE'</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>20</t>
+        <v>8</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (34%): 'proiecte Consiliul Local al Tinerilor' vs 'TITLUL II  BUNURI SI SERVICII'</t>
+          <t>unparseable cell 'VENITURI' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>10</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>80.02</t>
+        <v>8</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>est2027</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (35%): 'Cap 80.02 Alte servicii economice genera' vs 'Împrumuturi pentru persoane cu statut de'</t>
+          <t>unparseable cell 'Venituri operationale' in column est2027</t>
         </is>
       </c>
     </row>
@@ -29586,16 +29640,16 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (32%): 'investitii' vs 'TITLUL VII ALTE TRANSFERURI'</t>
+          <t>name mismatch vs nomenclator (34%): 'proiecte Consiliul Local al Tinerilor' vs 'TITLUL II  BUNURI SI SERVICII'</t>
         </is>
       </c>
     </row>
@@ -29611,16 +29665,16 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>80.02</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (33%): 'alte drepturi sociale' vs 'TITLUL II  BUNURI SI SERVICII'</t>
+          <t>name mismatch vs nomenclator (35%): 'Cap 80.02 Alte servicii economice genera' vs 'Împrumuturi pentru persoane cu statut de'</t>
         </is>
       </c>
     </row>
@@ -29640,37 +29694,37 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (44%): 'varsaminte la bugetul de stat aferent pe' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
+          <t>name mismatch vs nomenclator (32%): 'investitii' vs 'TITLUL VII ALTE TRANSFERURI'</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>11</v>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>unparseable cell "000'6" in column total_2026</t>
+          <t>name mismatch vs nomenclator (33%): 'alte drepturi sociale' vs 'TITLUL II  BUNURI SI SERVICII'</t>
         </is>
       </c>
     </row>
@@ -29686,48 +29740,48 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>20.02</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (38%): 'finantare complementara scoala' vs 'Reparatii curente'</t>
+          <t>name mismatch vs nomenclator (44%): 'varsaminte la bugetul de stat aferent pe' vs 'TITLUL I  CHELTUIELI DE PERSONAL'</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>14</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>20.02</t>
+        <v>11</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (44%): 'finantare complementara gradinita' vs 'Reparatii curente'</t>
+          <t>unparseable cell "000'6" in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -29736,16 +29790,16 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>20.02</t>
+          <t>31.02</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>duplicate of p14 with different values</t>
+          <t>name mismatch vs nomenclator (13%): '(materiale dendrologice, ingrasaminte, u' vs 'Venituri din dobanzi'</t>
         </is>
       </c>
     </row>
@@ -29761,16 +29815,16 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>70.02</t>
+          <t>35.02</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (32%): 'finantare de baza' vs 'Locuinte, servicii si dezvoltare publica'</t>
+          <t>name mismatch vs nomenclator (34%): 'iluminat public' vs 'Amenzi, penalitati si confiscari'</t>
         </is>
       </c>
     </row>
@@ -29786,73 +29840,73 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>15.02</t>
+          <t>35.02</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (34%): 'gradinita finantare de baza' vs 'Taxe pe servicii specifice'</t>
+          <t>name mismatch vs nomenclator (35%): 'materiale intretinere iluminat' vs 'Amenzi, penalitati si confiscari'</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>15</v>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>total</t>
+        <v>14</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>20.02</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>unparseable cell '1,042.00 642.00' in column total</t>
+          <t>name mismatch vs nomenclator (38%): 'finantare complementara scoala' vs 'Reparatii curente'</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>15</v>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>total</t>
+        <v>14</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>20.02</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>unparseable cell '1,195.00 854.00' in column total</t>
+          <t>name mismatch vs nomenclator (44%): 'finantare complementara gradinita' vs 'Reparatii curente'</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -29861,66 +29915,66 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>80.02</t>
+          <t>20.02</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (36%): 'finantare complementara' vs 'Actiuni generale economice, comerciale s'</t>
+          <t>duplicate of p14 with different values</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>15</v>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>total</t>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>70.02</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>unparseable cell '1,009.00 469.00' in column total</t>
+          <t>name mismatch vs nomenclator (32%): 'finantare de baza' vs 'Locuinte, servicii si dezvoltare publica'</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>15</v>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>total</t>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>15.02</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>unparseable cell '826.00 761.00' in column total</t>
+          <t>name mismatch vs nomenclator (34%): 'gradinita finantare de baza' vs 'Taxe pe servicii specifice'</t>
         </is>
       </c>
     </row>
@@ -29936,16 +29990,16 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>total_2026</t>
+          <t>total</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>unparseable cell '一' in column total_2026</t>
+          <t>unparseable cell '1,042.00 642.00' in column total</t>
         </is>
       </c>
     </row>
@@ -29961,41 +30015,41 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>total_2026</t>
+          <t>total</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>unparseable cell 'A' in column total_2026</t>
+          <t>unparseable cell '1,195.00 854.00' in column total</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>17</v>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>15</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>80.02</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>unparseable cell 'B' in column total_2026</t>
+          <t>name mismatch vs nomenclator (36%): 'finantare complementara' vs 'Actiuni generale economice, comerciale s'</t>
         </is>
       </c>
     </row>
@@ -30011,16 +30065,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>total_2026</t>
+          <t>total</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>unparseable cell 'II' in column total_2026</t>
+          <t>unparseable cell '1,009.00 469.00' in column total</t>
         </is>
       </c>
     </row>
@@ -30036,16 +30090,16 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>total_2026</t>
+          <t>total</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>unparseable cell 'ⅢII' in column total_2026</t>
+          <t>unparseable cell '826.00 761.00' in column total</t>
         </is>
       </c>
     </row>
@@ -30070,7 +30124,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>unparseable cell 'a' in column total_2026</t>
+          <t>unparseable cell '一' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -30095,57 +30149,57 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>unparseable cell 'b' in column total_2026</t>
+          <t>unparseable cell 'A' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>19</v>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>51.02.07</t>
+        <v>17</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (29%): 'AUTORITĂTI PUBLICE' vs 'Finanţarea studiilor de fezabilitate afe'</t>
+          <t>unparseable cell 'B' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>19</v>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>56</t>
+        <v>17</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (16%): '-r a t a n 1 2027' vs 'Titlul VIII PROIECTE CU FINANTARE DIN FO'</t>
+          <t>unparseable cell 'II' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -30155,47 +30209,47 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>warning</t>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>19</v>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>60</t>
+        <v>17</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>duplicate of p19 with different values</t>
+          <t>unparseable cell 'ⅢII' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>19</v>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>70.02.07</t>
+        <v>17</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (46%): 'LOCUINTE ŞI DEZVOLTARE PUBLICÃ, LOCUINTE' vs 'Alimantare cu gaze naturale in localitat'</t>
+          <t>unparseable cell 'a' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -30205,29 +30259,29 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>warning</t>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>19</v>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>56</t>
+        <v>17</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>duplicate of p19 with different values</t>
+          <t>unparseable cell 'b' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -30240,19 +30294,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>51.02.07</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>duplicate of p19 with different values</t>
+          <t>name mismatch vs nomenclator (29%): 'AUTORITĂTI PUBLICE' vs 'Finanţarea studiilor de fezabilitate afe'</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -30265,12 +30319,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>56</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>duplicate of p19 with different values</t>
+          <t>name mismatch vs nomenclator (16%): '-r a t a n 1 2027' vs 'Titlul VIII PROIECTE CU FINANTARE DIN FO'</t>
         </is>
       </c>
     </row>
@@ -30290,7 +30344,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -30311,23 +30365,23 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>12.02</t>
+          <t>70.02.07</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Alte impozite si taxe generale pe bunuri'</t>
+          <t>name mismatch vs nomenclator (46%): 'LOCUINTE ŞI DEZVOLTARE PUBLICÃ, LOCUINTE' vs 'Alimantare cu gaze naturale in localitat'</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -30336,16 +30390,16 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>12.02</t>
+          <t>56</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (43%): 'Sistem de avertizare audio-video si pano' vs 'Alte impozite si taxe generale pe bunuri'</t>
+          <t>duplicate of p19 with different values</t>
         </is>
       </c>
     </row>
@@ -30361,46 +30415,41 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>12.02</t>
+          <t>56</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>duplicate of p24 with different values</t>
+          <t>duplicate of p19 with different values</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>12.02</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>duplicate of p19 with different values</t>
         </is>
       </c>
     </row>
@@ -30410,34 +30459,34 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>24</v>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+        <v>19</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>56</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>unparseable cell 'IⅡI' in column total_2026</t>
+          <t>duplicate of p19 with different values</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -30445,17 +30494,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>24.02</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+          <t>12.02</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Alte impozite si taxe generale pe bunuri'</t>
         </is>
       </c>
     </row>
@@ -30475,19 +30519,19 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>30.02</t>
+          <t>12.02</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Venituri din proprietate'</t>
+          <t>name mismatch vs nomenclator (43%): 'Sistem de avertizare audio-video si pano' vs 'Alte impozite si taxe generale pe bunuri'</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -30500,12 +30544,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>30.02</t>
+          <t>12.02</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (46%): 'GRADINITA NR.18' vs 'Venituri din proprietate'</t>
+          <t>duplicate of p24 with different values</t>
         </is>
       </c>
     </row>
@@ -30525,7 +30569,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>30.02</t>
+          <t>12.02</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -30542,37 +30586,37 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C88" t="n">
         <v>24</v>
       </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>30.02</t>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Venituri din proprietate'</t>
+          <t>unparseable cell 'IⅡI' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V6_repair</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>info</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -30580,12 +30624,17 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>30.02</t>
+          <t>24.02</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>duplicate of p24 with different values</t>
+          <t>cell re-read from image (unverified transcription)</t>
         </is>
       </c>
     </row>
@@ -30610,19 +30659,19 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (38%): 'ALTE CHELTUIELI DE INVESTITII' vs 'Venituri din proprietate'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Venituri din proprietate'</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -30633,26 +30682,21 @@
           <t>30.02</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>total_2026</t>
-        </is>
-      </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>name mismatch vs nomenclator (46%): 'GRADINITA NR.18' vs 'Venituri din proprietate'</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V6_repair</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>info</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -30663,16 +30707,21 @@
           <t>30.02</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>total_2026</t>
+        </is>
+      </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (35%): 'Documentatie Refacere imprejmuire Gradin' vs 'Venituri din proprietate'</t>
+          <t>cell re-read from image (unverified transcription)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -30690,14 +30739,14 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>duplicate of p24 with different values</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Venituri din proprietate'</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -30715,19 +30764,19 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Venituri din proprietate'</t>
+          <t>duplicate of p24 with different values</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -30738,31 +30787,31 @@
           <t>30.02</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>total_2026</t>
-        </is>
-      </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>name mismatch vs nomenclator (38%): 'ALTE CHELTUIELI DE INVESTITII' vs 'Venituri din proprietate'</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B96" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V6_repair</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>info</t>
         </is>
       </c>
       <c r="C96" t="n">
         <v>24</v>
       </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>30.02</t>
+        </is>
+      </c>
       <c r="E96" t="inlineStr">
         <is>
           <t>total_2026</t>
@@ -30770,32 +30819,32 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>unparseable cell 'ⅡI' in column total_2026</t>
+          <t>cell re-read from image (unverified transcription)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B97" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C97" t="n">
         <v>24</v>
       </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>30.02</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>unparseable cell 'ⅡI' in column total_2026</t>
+          <t>name mismatch vs nomenclator (35%): 'Documentatie Refacere imprejmuire Gradin' vs 'Venituri din proprietate'</t>
         </is>
       </c>
     </row>
@@ -30805,64 +30854,69 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B98" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C98" t="n">
         <v>24</v>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>30.02</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>unparseable cell 'ⅡI' in column total_2026</t>
+          <t>duplicate of p24 with different values</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B99" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C99" t="n">
         <v>24</v>
       </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>30.02</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>unparseable cell 'ⅡI' in column total_2026</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Venituri din proprietate'</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B100" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V6_repair</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>info</t>
         </is>
       </c>
       <c r="C100" t="n">
         <v>24</v>
       </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>30.02</t>
+        </is>
+      </c>
       <c r="E100" t="inlineStr">
         <is>
           <t>total_2026</t>
@@ -30870,7 +30924,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>unparseable cell 'ⅡI' in column total_2026</t>
+          <t>cell re-read from image (unverified transcription)</t>
         </is>
       </c>
     </row>
@@ -30895,7 +30949,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>unparseable cell 'IⅡI' in column total_2026</t>
+          <t>unparseable cell 'ⅡI' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -30920,7 +30974,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>unparseable cell 'I' in column total_2026</t>
+          <t>unparseable cell 'ⅡI' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -30977,50 +31031,50 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C105" t="n">
         <v>24</v>
       </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>10.02</t>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Cheltuieli salariale in natura'</t>
+          <t>unparseable cell 'ⅡI' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C106" t="n">
         <v>24</v>
       </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>10.02</t>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (44%): 'LICEUL CU PROGRAM SPORTIV' vs 'Cheltuieli salariale in natura'</t>
+          <t>unparseable cell 'IⅡI' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -31030,44 +31084,39 @@
           <t>V7_hygiene</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>warning</t>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C107" t="n">
         <v>24</v>
       </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>10.02</t>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>duplicate of p24 with different values</t>
+          <t>unparseable cell 'I' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>V6_repair</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>info</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C108" t="n">
         <v>24</v>
       </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>10.02</t>
-        </is>
-      </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>total_2026</t>
@@ -31075,32 +31124,32 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>unparseable cell 'ⅡI' in column total_2026</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>V2_name</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>warning</t>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="C109" t="n">
         <v>24</v>
       </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>10.02</t>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>total_2026</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (0%): '' vs 'Cheltuieli salariale in natura'</t>
+          <t>unparseable cell 'ⅡI' in column total_2026</t>
         </is>
       </c>
     </row>
@@ -31125,14 +31174,14 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (54%): 'ALTE CHELTUIELI DE INVESTITII' vs 'Cheltuieli salariale in natura'</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Cheltuieli salariale in natura'</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -31150,19 +31199,19 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>duplicate of p24 with different values</t>
+          <t>name mismatch vs nomenclator (44%): 'LICEUL CU PROGRAM SPORTIV' vs 'Cheltuieli salariale in natura'</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -31173,26 +31222,21 @@
           <t>10.02</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>total_2026</t>
-        </is>
-      </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>duplicate of p24 with different values</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V6_repair</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>info</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -31203,9 +31247,14 @@
           <t>10.02</t>
         </is>
       </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>total_2026</t>
+        </is>
+      </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (39%): 'Statie dedurizare apa' vs 'Cheltuieli salariale in natura'</t>
+          <t>cell re-read from image (unverified transcription)</t>
         </is>
       </c>
     </row>
@@ -31237,7 +31286,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
+          <t>V2_name</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -31255,19 +31304,19 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>duplicate of p24 with different values</t>
+          <t>name mismatch vs nomenclator (54%): 'ALTE CHELTUIELI DE INVESTITII' vs 'Cheltuieli salariale in natura'</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>V6_repair</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -31278,31 +31327,31 @@
           <t>10.02</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>total_2026</t>
-        </is>
-      </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>cell re-read from image (unverified transcription)</t>
+          <t>duplicate of p24 with different values</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B117" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V6_repair</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>info</t>
         </is>
       </c>
       <c r="C117" t="n">
         <v>24</v>
       </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>10.02</t>
+        </is>
+      </c>
       <c r="E117" t="inlineStr">
         <is>
           <t>total_2026</t>
@@ -31310,64 +31359,64 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>unparseable cell 'I' in column total_2026</t>
+          <t>cell re-read from image (unverified transcription)</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B118" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C118" t="n">
         <v>24</v>
       </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>10.02</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>unparseable cell 'II' in column total_2026</t>
+          <t>name mismatch vs nomenclator (39%): 'Statie dedurizare apa' vs 'Cheltuieli salariale in natura'</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>V7_hygiene</t>
-        </is>
-      </c>
-      <c r="B119" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="C119" t="n">
         <v>24</v>
       </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>total_2026</t>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>10.02</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>unparseable cell 'ⅡI' in column total_2026</t>
+          <t>name mismatch vs nomenclator (0%): '' vs 'Cheltuieli salariale in natura'</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V7_hygiene</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -31376,64 +31425,194 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>70.02</t>
+          <t>10.02</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (36%): 'Documentatie PUZ Amenajare cale de acces' vs 'Locuinte, servicii si dezvoltare publica'</t>
+          <t>duplicate of p24 with different values</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>V2_name</t>
+          <t>V6_repair</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>info</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
           <t>10.02</t>
         </is>
       </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>total_2026</t>
+        </is>
+      </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>name mismatch vs nomenclator (30%): 'Placa vibro-compactoare' vs 'Cheltuieli salariale in natura'</t>
+          <t>cell re-read from image (unverified transcription)</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>24</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>total_2026</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>unparseable cell 'I' in column total_2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>24</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>total_2026</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>unparseable cell 'II' in column total_2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>V7_hygiene</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>24</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>total_2026</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>unparseable cell 'ⅡI' in column total_2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
           <t>V2_name</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
+      <c r="B125" t="inlineStr">
         <is>
           <t>warning</t>
         </is>
       </c>
-      <c r="C122" t="n">
+      <c r="C125" t="n">
         <v>30</v>
       </c>
-      <c r="D122" t="inlineStr">
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>70.02</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>name mismatch vs nomenclator (36%): 'Documentatie PUZ Amenajare cale de acces' vs 'Locuinte, servicii si dezvoltare publica'</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>30</v>
+      </c>
+      <c r="D126" t="inlineStr">
         <is>
           <t>10.02</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr">
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>name mismatch vs nomenclator (30%): 'Placa vibro-compactoare' vs 'Cheltuieli salariale in natura'</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>V2_name</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>30</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>10.02</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
         <is>
           <t>name mismatch vs nomenclator (0%): '' vs 'Cheltuieli salariale in natura'</t>
         </is>
@@ -31486,7 +31665,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4">
@@ -31506,7 +31685,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>73</v>
+        <v>71.8</v>
       </c>
     </row>
     <row r="6">
@@ -31516,7 +31695,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
@@ -31526,7 +31705,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8">

</xml_diff>